<commit_message>
Added conditional hooks. Added extent,allure reports,log4j.Added methods in element utils.
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData/TestData.xlsx
+++ b/src/test/resources/TestData/TestData.xlsx
@@ -8,14 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lingesh Raja\git\Ds_AlGO_BDD\src\test\resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBEDA250-745E-4919-94D4-03BD50320E65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3FA0466-8D58-4A90-82EF-E40DA5A8D872}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="LoginCredentials" sheetId="3" r:id="rId1"/>
-    <sheet name="SuccessfulRegistration" sheetId="1" r:id="rId2"/>
-    <sheet name="TryEditor" sheetId="5" r:id="rId3"/>
+    <sheet name="TestData" sheetId="3" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
   <si>
     <t>sdfglkjh@24</t>
   </si>
@@ -72,31 +70,34 @@
   </si>
   <si>
     <t>print("Hello")</t>
+  </si>
+  <si>
+    <t>CodeType</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>ExpectedOutput</t>
+  </si>
+  <si>
+    <t>NameError: name 'System' is not defined on line 1</t>
+  </si>
+  <si>
+    <t>Hello</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Consolas"/>
-      <family val="3"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF008000"/>
-      <name val="Consolas"/>
-      <family val="3"/>
     </font>
     <font>
       <b/>
@@ -112,14 +113,6 @@
       <color rgb="FF000000"/>
       <name val="Consolas"/>
       <family val="3"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -145,25 +138,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -442,173 +428,92 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{358C323C-EFB0-421A-987A-331ECC3C90CA}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="2" width="16.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.81640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.08984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="56.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.08984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="43.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>17</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>9</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B3" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C3" t="s">
         <v>0</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="1"/>
-      <c r="D3" s="1"/>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B4" s="1"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="1"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="1"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="1"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" s="1"/>
-      <c r="D8" s="1"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" s="1"/>
-      <c r="D9" s="1"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="3"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="3"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" s="3"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="3"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" s="3"/>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A17" s="3"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09880E84-3817-4B86-8851-21FADE6B3A0D}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C1" s="5" t="s">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="F5" t="s">
         <v>14</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>